<commit_message>
Build Q2475 Kubernetes Windows task
</commit_message>
<xml_diff>
--- a/task/任务规格转化.xlsx
+++ b/task/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="Ra4efb9a5be394325"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R0aaf8a8385be41c9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -314,7 +314,7 @@
         <x:v>输入来源</x:v>
       </x:c>
       <x:c r="B5" s="5" t="str">
-        <x:v>支付平台准备的虚构现行Service、后端地址和发布规则</x:v>
+        <x:v>支付平台从现行发布清单和本次维护窗登记中整理的Service、后端地址和发布规则</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">

</xml_diff>